<commit_message>
6 junio 2020 v2
</commit_message>
<xml_diff>
--- a/_downloads/ecb565b050d60b24d8694a8a1c9d2cf7/3. Indicadores de desempeño.xlsx
+++ b/_downloads/ecb565b050d60b24d8694a8a1c9d2cf7/3. Indicadores de desempeño.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\ADMINISTRACIÓN DE INVERSIONES\Teoría moderna de portafolios de inversión\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22ADF608-C440-454E-A702-ADF66E6DE6B8}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75B5D297-063A-492E-85BD-0A905D94294D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="47">
   <si>
     <t>Fecha</t>
   </si>
@@ -277,6 +277,12 @@
   </si>
   <si>
     <t>Por cada unidad de riesgo sistemático, el portafolio tuvo un exceso de rentabilidad de 3,88% por año.</t>
+  </si>
+  <si>
+    <t>Por cada 1% de riesgo que se toma el portafolio entrega 0,0061% de rendimiento en exceso a la tasa libre de riesgo.</t>
+  </si>
+  <si>
+    <t>Por cada 1% de riesgo que se toma el portafolio entrega 0,0965% de rendimiento en exceso a la tasa libre de riesgo.</t>
   </si>
 </sst>
 </file>
@@ -895,13 +901,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3970,14 +3976,14 @@
       <c r="F1" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="G1" s="32" t="s">
+      <c r="G1" s="33" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="32"/>
-      <c r="I1" s="32"/>
-      <c r="J1" s="32"/>
-      <c r="K1" s="32"/>
-      <c r="L1" s="32"/>
+      <c r="H1" s="33"/>
+      <c r="I1" s="33"/>
+      <c r="J1" s="33"/>
+      <c r="K1" s="33"/>
+      <c r="L1" s="33"/>
       <c r="M1" s="19" t="s">
         <v>26</v>
       </c>
@@ -4961,10 +4967,10 @@
         <f t="shared" si="1"/>
         <v>8.1942907070158694E-4</v>
       </c>
-      <c r="N19" s="33" t="s">
+      <c r="N19" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="O19" s="33"/>
+      <c r="O19" s="34"/>
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
@@ -5015,7 +5021,7 @@
       <c r="N20" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="O20" s="34">
+      <c r="O20" s="32">
         <f>+(O8-Q16)/O9</f>
         <v>6.100681919896038E-3</v>
       </c>
@@ -5024,6 +5030,9 @@
       </c>
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
+      <c r="Y20" s="1" t="s">
+        <v>45</v>
+      </c>
       <c r="AG20" s="11"/>
     </row>
     <row r="21" spans="1:33" x14ac:dyDescent="0.2">
@@ -5072,7 +5081,7 @@
       <c r="N21" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="O21" s="34">
+      <c r="O21" s="32">
         <f>+(O8-Q16)/O10</f>
         <v>1.5526778410412966E-4</v>
       </c>
@@ -5949,10 +5958,10 @@
         <f t="shared" si="1"/>
         <v>5.8983195508717815E-4</v>
       </c>
-      <c r="N38" s="33" t="s">
+      <c r="N38" s="34" t="s">
         <v>15</v>
       </c>
-      <c r="O38" s="33"/>
+      <c r="O38" s="34"/>
     </row>
     <row r="39" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
@@ -6000,7 +6009,7 @@
       <c r="N39" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="O39" s="34">
+      <c r="O39" s="32">
         <f>+(O33-O16)/O34</f>
         <v>9.6460250735401903E-2</v>
       </c>
@@ -6012,6 +6021,9 @@
       </c>
       <c r="R39" s="3"/>
       <c r="S39" s="3"/>
+      <c r="Z39" s="1" t="s">
+        <v>46</v>
+      </c>
       <c r="AH39" s="11"/>
     </row>
     <row r="40" spans="1:36" x14ac:dyDescent="0.2">
@@ -6060,7 +6072,7 @@
       <c r="N40" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="O40" s="34">
+      <c r="O40" s="32">
         <f>+(O33-O16)/O10</f>
         <v>3.8816946026032424E-2</v>
       </c>

</xml_diff>